<commit_message>
feat: auto-populate API keys from .env.local via Vite env vars
Store DEFAULT_SETTINGS now reads VITE_* environment variables so that
keys defined in .env.local (e.g. VITE_GOOGLE_PLACES_API_KEY) are
pre-loaded into settings on first run without manual UI entry.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/IvoireGrowthScan-V4-Dev.xlsx
+++ b/assets/IvoireGrowthScan-V4-Dev.xlsx
@@ -413,7 +413,7 @@
     <t>API + Script Python</t>
   </si>
   <si>
-    <t>SEMrush API ou Ahrefs API</t>
+    <t>SimilarWeb, SEMrush API ou Ahrefs API</t>
   </si>
   <si>
     <t>Sim — SEMrush ($139–499/mês) ou Ahrefs ($99–399/mês)</t>
@@ -2940,7 +2940,7 @@
       <c r="E4" s="12" t="s">
         <v>132</v>
       </c>
-      <c r="F4" s="12" t="s">
+      <c r="F4" s="13" t="s">
         <v>133</v>
       </c>
       <c r="G4" s="12" t="s">

</xml_diff>